<commit_message>
added methods of apply
</commit_message>
<xml_diff>
--- a/docs/countries.xlsx
+++ b/docs/countries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramtin\Documents\Projects\personal\resume\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7A3052-A2A6-474F-86DC-6C8E6493204F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51AE3B6-5776-4055-A3EB-72D3E46236BF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17505" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1097,7 +1097,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="#,##0.#"/>
+    <numFmt numFmtId="164" formatCode="#,##0.#"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1175,10 +1175,10 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>

</xml_diff>